<commit_message>
Gauge lights, Hurst T-handle grip, dash detail scripts and cost update
- Wiring: gauge lamps lit from the NAV rocker or a second pole on the
  light bar rotary through two 1N5408 diodes, all inside the dash
  (schematic page, control SVG and PDF).
- Grip: real Hurst 1530040 T-handle on an M16 x 1.5 stud with a 316
  nylon-insert lock nut and 1/4 in cross pin, rated 450 lb at the handle;
  four new checks in structure.py / Structural_Checks (stick and frame
  still 600 lb). BOM, build guide, ledger, README and Getting Started.
- BOM: 2-pole light bar rotary, 13th wire colour, 4 diodes, T-handle.
- Marketing: cost figures and calculator match the BOM.
- Fusion scripts: WhiteGauges fixes, GaugeDials, ConsoleLabels, TGrip.
- Package zip refreshed; .gitignore skips .vscode.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/StraddleDart_rev7/BOM_rev7.xlsx
+++ b/StraddleDart_rev7/BOM_rev7.xlsx
@@ -633,7 +633,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="23.85" customHeight="1" s="31">
       <c r="A4" s="34" t="inlineStr">
         <is>
@@ -882,7 +881,6 @@
       <c r="D18" s="41" t="n"/>
       <c r="E18" s="41" t="n"/>
     </row>
-    <row r="19"/>
     <row r="20" ht="15" customHeight="1" s="31">
       <c r="A20" s="33" t="inlineStr">
         <is>
@@ -937,7 +935,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="23.85" customHeight="1" s="31">
       <c r="A4" s="49" t="inlineStr">
         <is>
@@ -1708,7 +1705,6 @@
         </is>
       </c>
     </row>
-    <row r="24"/>
     <row r="25" ht="15" customHeight="1" s="31">
       <c r="A25" s="38" t="inlineStr">
         <is>
@@ -1808,7 +1804,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="23.85" customHeight="1" s="31">
       <c r="A4" s="49" t="inlineStr">
         <is>
@@ -3175,7 +3170,6 @@
       <c r="I39" s="52" t="n"/>
       <c r="J39" s="50" t="n"/>
     </row>
-    <row r="40"/>
     <row r="41" ht="15" customHeight="1" s="31">
       <c r="A41" s="38" t="inlineStr">
         <is>
@@ -3279,7 +3273,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="23.85" customHeight="1" s="31">
       <c r="A4" s="49" t="inlineStr">
         <is>
@@ -5651,12 +5644,12 @@
     <row r="69">
       <c r="A69" s="50" t="inlineStr">
         <is>
-          <t>Grip (hand-hold), Hurst style</t>
+          <t>Grip (hand-hold), Hurst T-handle</t>
         </is>
       </c>
       <c r="B69" s="50" t="inlineStr">
         <is>
-          <t>1-1/8 in 316 SS rod, bent, welded to a 3 x 2 x 1/4 in 316 base plate; 4 x 1/4 in 316 bolts through the console top and both rail walls with crush tubes, Tef-Gel and a gasket; 1-7/8 in white ball knob</t>
+          <t>1-1/8 in 316 SS rod, cold-drawn (A276 Condition B), bent, welded to a 3 x 2 x 1/4 in 316 base plate; 4 x 1/4 in 316 bolts through the console top and both rail walls with crush tubes, Tef-Gel and a gasket; Hurst 1530040 universal T-handle, polished cast aluminium (new about $62-68, or used on eBay), bar across the boat, threaded straight onto an M16 x 1.5 stud turned on the stick end (no adapter), 316 M16 x 1.5 nylon-insert lock nut under the neck, 1/4 in 316 cross pin</t>
         </is>
       </c>
       <c r="C69" s="51" t="n">
@@ -5668,7 +5661,7 @@
         </is>
       </c>
       <c r="E69" s="53" t="n">
-        <v>85</v>
+        <v>140</v>
       </c>
       <c r="F69" s="54">
         <f>C69*E69</f>
@@ -5685,7 +5678,7 @@
       <c r="I69" s="52" t="n"/>
       <c r="J69" s="50" t="inlineStr">
         <is>
-          <t>Stainless cannot be welded to the 6061 rail; sized for 600 lbf (factor 2.2 on yield); knob position from drv_reach</t>
+          <t>Stainless cannot be welded to the 6061 rail; stick and plate sized for 600 lbf; the Hurst handle on its pinned M16 stud is rated 450 lb (Structural_Checks); T-handle position from drv_reach. The Hurst handle is a shift knob: the pin stops a hard sideways pull from unscrewing it. Pull-test the finished grip before use</t>
         </is>
       </c>
     </row>
@@ -5898,7 +5891,7 @@
       </c>
       <c r="B75" s="50" t="inlineStr">
         <is>
-          <t>2 sealed OFF-LO-MED-HI rotary switches (light bar, searchlight) + sealed NAV-OFF-ANCHOR rocker; DT12 connector</t>
+          <t>2 sealed OFF-LO-MED-HI rotary switches (light bar 2-pole, its second pole lights the gauges; searchlight) + sealed NAV-OFF-ANCHOR rocker; DT12 connector</t>
         </is>
       </c>
       <c r="C75" s="51" t="n">
@@ -5910,7 +5903,7 @@
         </is>
       </c>
       <c r="E75" s="53" t="n">
-        <v>85</v>
+        <v>95</v>
       </c>
       <c r="F75" s="54">
         <f>C75*E75</f>
@@ -6377,16 +6370,16 @@
     <row r="87">
       <c r="A87" s="50" t="inlineStr">
         <is>
-          <t>Primary 18 AWG tinned marine, 12 colours</t>
+          <t>Primary 18 AWG tinned marine, 13 colours</t>
         </is>
       </c>
       <c r="B87" s="50" t="inlineStr">
         <is>
-          <t>Key, kill, gauges, sensors (tach dark gray, temp tan, fuel pink, trouble brown-white), dimmer and relay signals, bilge, pump; 25 ft spools</t>
+          <t>Key, kill, gauges, sensors (tach dark gray, temp tan, fuel pink, trouble brown-white, gauge lights blue-yellow), dimmer and relay signals, bilge, pump; 25 ft spools</t>
         </is>
       </c>
       <c r="C87" s="51" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D87" s="52" t="inlineStr">
         <is>
@@ -6501,7 +6494,7 @@
       </c>
       <c r="B90" s="50" t="inlineStr">
         <is>
-          <t>5 x 12 V 40 A relays (start, EFI main, fuel pump, nav, anchor) + 2 x 1N5408 diodes; 2 x IP67 20 A PWM dimmers with 3-wire remote input</t>
+          <t>5 x 12 V 40 A relays (start, EFI main, fuel pump, nav, anchor) + 4 x 1N5408 diodes (2 anchor coil, 2 gauge lights); 2 x IP67 20 A PWM dimmers with 3-wire remote input</t>
         </is>
       </c>
       <c r="C90" s="51" t="n">
@@ -6940,7 +6933,6 @@
       <c r="I100" s="52" t="n"/>
       <c r="J100" s="50" t="n"/>
     </row>
-    <row r="101"/>
     <row r="102">
       <c r="A102" s="38" t="inlineStr">
         <is>

</xml_diff>